<commit_message>
sua doi chia tu vung phu hop
</commit_message>
<xml_diff>
--- a/chu_de.xlsx
+++ b/chu_de.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BRAVO 15\Downloads\game tieng trung hsk 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413335FD-18D5-44B3-9569-843BF054810A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32566B7C-64D2-4626-ABBF-C7A30D9EB769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Chủ đề" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="50">
   <si>
     <t>Chủ đề</t>
   </si>
@@ -34,7 +34,76 @@
     <t>Gợi ý hoạt động</t>
   </si>
   <si>
-    <t>1. Con người &amp; Các mối quan hệ</t>
+    <t>1. Con người &amp; Các mối quan hệ (Phần 1)</t>
+  </si>
+  <si>
+    <t>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</t>
+  </si>
+  <si>
+    <t>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</t>
+  </si>
+  <si>
+    <t>1. Con người &amp; Các mối quan hệ (Phần 2)</t>
+  </si>
+  <si>
+    <t>2. Cơ thể &amp; Sức khỏe</t>
+  </si>
+  <si>
+    <t>3. Cảm xúc &amp; Thái độ</t>
+  </si>
+  <si>
+    <t>4. Tư duy &amp; Nhận thức</t>
+  </si>
+  <si>
+    <t>5. Đời sống sinh hoạt</t>
+  </si>
+  <si>
+    <t>6. Đồ vật &amp; Công cụ</t>
+  </si>
+  <si>
+    <t>7. Địa điểm &amp; Nơi chốn</t>
+  </si>
+  <si>
+    <t>8. Giao thông &amp; Di chuyển</t>
+  </si>
+  <si>
+    <t>9. Không gian &amp; Vị trí</t>
+  </si>
+  <si>
+    <t>10. Thời gian (Phần 1)</t>
+  </si>
+  <si>
+    <t>10. Thời gian (Phần 2)</t>
+  </si>
+  <si>
+    <t>12. Công việc &amp; Nghề nghiệp</t>
+  </si>
+  <si>
+    <t>13. Miêu tả &amp; Đánh giá</t>
+  </si>
+  <si>
+    <t>14. Số lượng &amp; Đo lường (Phần 1)</t>
+  </si>
+  <si>
+    <t>14. Số lượng &amp; Đo lường (Phần 2)</t>
+  </si>
+  <si>
+    <t>14. Số lượng &amp; Đo lường (Phần 3)</t>
+  </si>
+  <si>
+    <t>15. Công cụ ngữ pháp &amp; Cấu trúc (Phần 1)</t>
+  </si>
+  <si>
+    <t>15. Công cụ ngữ pháp &amp; Cấu trúc (Phần 2)</t>
+  </si>
+  <si>
+    <t>15. Công cụ ngữ pháp &amp; Cấu trúc (Phần 3)</t>
+  </si>
+  <si>
+    <t>16. Tự nhiên</t>
+  </si>
+  <si>
+    <t>17. Đồ ăn &amp; Thức uống</t>
   </si>
   <si>
     <t>1. 爸爸
@@ -54,35 +123,41 @@
 15. 男
 16. 男朋友
 17. 你
-18. 你们
-19. 您
-20. 女
-21. 女儿
-22. 女朋友
-23. 女士
-24. 朋友
-25. 人
-26. 谁
-27. 他
-28. 他们
-29. 它
-30. 它们
-31. 她们
-32. 同学
-33. 我
-34. 我们
-35. 先生
-36. 小朋友
-37. 她</t>
-  </si>
-  <si>
-    <t>Sử dụng trong các buổi khởi động (Warm-up) hoặc ôn tập sau bài học (Review).</t>
-  </si>
-  <si>
-    <t>Chia lớp thành 2 đội (Trộm &amp; Cảnh sát). Mỗi lượt đi yêu cầu trả lời đúng từ vựng để được di chuyển.</t>
-  </si>
-  <si>
-    <t>4. Tư duy &amp; Nhận thức</t>
+18. 你们</t>
+  </si>
+  <si>
+    <t>1. 您
+2. 女
+3. 女儿
+4. 女朋友
+5. 女士
+6. 朋友
+7. 人
+8. 谁
+9. 他
+10. 他们
+11. 它
+12. 它们
+13. 她们
+14. 同学
+15. 我
+16. 我们
+17. 先生
+18. 小朋友
+19. 她</t>
+  </si>
+  <si>
+    <t>1. 病
+2. 病人
+3. 看病
+4. 生病
+5. 药</t>
+  </si>
+  <si>
+    <t>1. 爱
+2. 高兴
+3. 觉得
+4. 喜欢</t>
   </si>
   <si>
     <t>1. 读
@@ -104,9 +179,6 @@
 17. 学
 18. 学习
 19. 知道</t>
-  </si>
-  <si>
-    <t>5. Đời sống sinh hoạt</t>
   </si>
   <si>
     <t>1. 唱
@@ -131,9 +203,6 @@
 20. 做饭</t>
   </si>
   <si>
-    <t>6. Đồ vật &amp; Công cụ</t>
-  </si>
-  <si>
     <t>1. 杯
 2. 杯子
 3. 电话
@@ -154,9 +223,6 @@
 18. 字
 19. 汉语
 20. 汉字</t>
-  </si>
-  <si>
-    <t>7. Địa điểm &amp; Nơi chốn</t>
   </si>
   <si>
     <t>1. 超市
@@ -183,9 +249,6 @@
 22. 北京</t>
   </si>
   <si>
-    <t>8. Giao thông &amp; Di chuyển</t>
-  </si>
-  <si>
     <t>1. 车
 2. 出租车
 3. 到
@@ -196,9 +259,6 @@
 8. 来
 9. 去
 10. 坐</t>
-  </si>
-  <si>
-    <t>9. Không gian &amp; Vị trí</t>
   </si>
   <si>
     <t>1. 边
@@ -215,39 +275,35 @@
 12. 这个</t>
   </si>
   <si>
-    <t>10. Thời gian</t>
-  </si>
-  <si>
     <t>1. 白天
 2. 点
 3. 分
 4. 分钟
-5. 今年
-6. 今天
-7. 明年
-8. 明天
-9. 年
-10. 去年
-11. 日
-12. 上午
-13. 时候
-14. 时间
-15. 晚
-16. 晚上
-17. 下午
-18. 现在
-19. 小时
-20. 星期
-21. 星期日
-22. 星期天
-23. 月
-24. 早
-25. 早上
-26. 中午
-27. 昨天</t>
-  </si>
-  <si>
-    <t>12. Công việc &amp; Nghề nghiệp</t>
+5. 年
+6. 去年
+7. 日
+8. 上午
+9. 时候
+10. 时间
+11. 晚</t>
+  </si>
+  <si>
+    <t>1. 今年
+2. 今天
+3. 明年
+4. 明天
+5. 晚上
+6. 下午
+7. 现在
+8. 小时
+9. 星期
+10. 星期日
+11. 星期天
+12. 月
+13. 早
+14. 早上
+15. 中午
+16. 昨天</t>
   </si>
   <si>
     <t>1. 大学生
@@ -265,9 +321,6 @@
 13. 医
 14. 医生
 15. 中学生</t>
-  </si>
-  <si>
-    <t>13. Miêu tả &amp; Đánh giá</t>
   </si>
   <si>
     <t>1. 大
@@ -290,9 +343,6 @@
 18. 真</t>
   </si>
   <si>
-    <t>14. Số lượng &amp; Đo lường</t>
-  </si>
-  <si>
     <t>1. 八
 2. 百
 3. 半
@@ -304,33 +354,34 @@
 9. 号
 10. 几
 11. 斤
-12. 九
-13. 口
-14. 块
-15. 两
-16. 零
-17. 六
-18. 七
-19. 千
-20. 三
-21. 十
-22. 四
-23. 岁
-24. 五
-25. 些
-26. 一
-27. 一半
-28. 一下
-29. 一点儿
-30. 一些
-31. 有
-32. 有的
-33. 有点儿
-34. 有些
-35. 只</t>
-  </si>
-  <si>
-    <t>15. Công cụ ngữ pháp &amp; Cấu trúc</t>
+12. 九</t>
+  </si>
+  <si>
+    <t>1. 口
+2. 块
+3. 两
+4. 零
+5. 六
+6. 七
+7. 千
+8. 三
+9. 十
+10. 四
+11. 岁
+12. 五</t>
+  </si>
+  <si>
+    <t>1. 些
+2. 一
+3. 一半
+4. 一下
+5. 一点儿
+6. 一些
+7. 有
+8. 有的
+9. 有点儿
+10. 有些
+11. 只</t>
   </si>
   <si>
     <t>1. 吧
@@ -352,32 +403,43 @@
 17. 没有
 18. 哪
 19. 哪里
-20. 哪儿
-21. 那
-22. 那里
-23. 那儿
-24. 呢
-25. 能
-26. 你好
-27. 请
-28. 什么
-29. 是
-30. 太
-31. 喂
-32. 谢谢
-33. 要
-34. 也
-35. 再
-36. 再见
-37. 在
-38. 怎么
-39. 怎么样
-40. 这
-41. 这些
-42. 正在</t>
-  </si>
-  <si>
-    <t>17. Đồ ăn &amp; Thức uống</t>
+20. 那里
+21. 那儿</t>
+  </si>
+  <si>
+    <t>1. 呢
+2. 能
+3. 你好
+4. 请
+5. 什么
+6. 是
+7. 太
+8. 喂
+9. 谢谢
+10. 要
+11. 也
+12. 再
+13. 再见
+14. 在
+15. 怎么
+16. 怎么样
+17. 这
+18. 这些
+19. 正在</t>
+  </si>
+  <si>
+    <t>1. 哪儿
+2. 那</t>
+  </si>
+  <si>
+    <t>1. 狗
+2. 猫
+3. 水
+4. 天
+5. 天气
+6. 下雨
+7. 雪
+8. 雨</t>
   </si>
   <si>
     <t>1. 包子
@@ -775,14 +837,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="30.796875" customWidth="1"/>
-    <col min="2" max="2" width="20.796875" customWidth="1"/>
-    <col min="3" max="3" width="40.796875" customWidth="1"/>
-    <col min="4" max="4" width="60.796875" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -798,193 +854,318 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="312" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="327.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="296.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="78" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="312" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="296.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="327.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="312" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="312" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="358.8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="343.2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="156" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="280.8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="312" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="296.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>19</v>
       </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="234" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="202.8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="358.8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="280.8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="B19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="312" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>25</v>
       </c>
-      <c r="C11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="B21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="265.2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>27</v>
       </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" t="s">
-        <v>7</v>
+      <c r="B23" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A14 A2 C2:D2 A3 C3:D3 A4 C4:D4 A5 C5:D5 A6 C6:D6 A7 C7:D7 A8 C8:D8 A9 C9:D9 A10 C10:D10 A11 C11:D11 A12 C12:D12 A13 C13:D13 C14:D14" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 A23 A2 C2:D2 A3 C3:D3 A4 C4:D4 A5 C5:D5 A6 C6:D6 A7 C7:D7 A8 C8:D8 A9 C9:D9 A10 C10:D10 A11 C11:D11 A12 C12:D12 A13 C13:D13 A14 C14:D14 A15 C15:D15 A16 C16:D16 A17 C17:D17 A18 C18:D18 A19 C19:D19 A20 C20:D20 A21 C21:D21 A22 C22:D22 C23:D23" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>